<commit_message>
Update KPI Summary Excel file and remove temporary backup
</commit_message>
<xml_diff>
--- a/excel/KPI_Summary.xlsx
+++ b/excel/KPI_Summary.xlsx
@@ -1,20 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\btheard\projects\batchbridge\excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBF96C97-6E72-47F8-868A-8719C7334740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="16663" windowHeight="8743" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="KPI_Summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Monthly_Metrics" sheetId="2" r:id="rId2"/>
+    <sheet name="Top_Countries" sheetId="3" r:id="rId3"/>
+    <sheet name="Dashboard" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>Metric</t>
   </si>
@@ -35,15 +57,85 @@
   </si>
   <si>
     <t>Repeat Customer Rate</t>
+  </si>
+  <si>
+    <t>total_transactions</t>
+  </si>
+  <si>
+    <t>total_sales</t>
+  </si>
+  <si>
+    <t>YearMonth</t>
+  </si>
+  <si>
+    <t>Sweden</t>
+  </si>
+  <si>
+    <t>Belgium</t>
+  </si>
+  <si>
+    <t>Switzerland</t>
+  </si>
+  <si>
+    <t>Spain</t>
+  </si>
+  <si>
+    <t>Australia</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>EIRE</t>
+  </si>
+  <si>
+    <t>Netherlands</t>
+  </si>
+  <si>
+    <t>United Kingdom</t>
+  </si>
+  <si>
+    <t>SalesAmount</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>AOV</t>
+  </si>
+  <si>
+    <t>Repeat Rate</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,21 +162,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -122,7 +227,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -156,6 +261,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -190,9 +296,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -365,11 +472,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="19.84375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -377,15 +487,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
-        <v>8911407.903999999</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>8911407.9039999992</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -393,7 +503,7 @@
         <v>18532</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -401,23 +511,351 @@
         <v>4338</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5">
-        <v>480.8659563997409</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+        <v>480.86595639974092</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0.6558321807284463</v>
+        <v>0.65583218072844629</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F520B5FF-16F3-4FC3-891E-A1847FEC4EE0}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="17.765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.765625" customWidth="1"/>
+    <col min="3" max="3" width="15.15234375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A2" s="1">
+        <v>40513</v>
+      </c>
+      <c r="B2">
+        <v>572713.89</v>
+      </c>
+      <c r="C2">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A3" s="1">
+        <v>40544</v>
+      </c>
+      <c r="B3">
+        <v>569445.04</v>
+      </c>
+      <c r="C3">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A4" s="1">
+        <v>40575</v>
+      </c>
+      <c r="B4">
+        <v>447137.35</v>
+      </c>
+      <c r="C4">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A5" s="1">
+        <v>40603</v>
+      </c>
+      <c r="B5">
+        <v>595500.76</v>
+      </c>
+      <c r="C5">
+        <v>1321</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A6" s="1">
+        <v>40634</v>
+      </c>
+      <c r="B6">
+        <v>469200.36099999998</v>
+      </c>
+      <c r="C6">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A7" s="1">
+        <v>40664</v>
+      </c>
+      <c r="B7">
+        <v>678594.56000000006</v>
+      </c>
+      <c r="C7">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A8" s="1">
+        <v>40695</v>
+      </c>
+      <c r="B8">
+        <v>661213.69000000006</v>
+      </c>
+      <c r="C8">
+        <v>1393</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A9" s="1">
+        <v>40725</v>
+      </c>
+      <c r="B9">
+        <v>600091.01100000006</v>
+      </c>
+      <c r="C9">
+        <v>1331</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A10" s="1">
+        <v>40756</v>
+      </c>
+      <c r="B10">
+        <v>645343.9</v>
+      </c>
+      <c r="C10">
+        <v>1280</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A11" s="1">
+        <v>40787</v>
+      </c>
+      <c r="B11">
+        <v>952838.38199999998</v>
+      </c>
+      <c r="C11">
+        <v>1755</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A12" s="1">
+        <v>40817</v>
+      </c>
+      <c r="B12">
+        <v>1039318.79</v>
+      </c>
+      <c r="C12">
+        <v>1929</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A13" s="1">
+        <v>40848</v>
+      </c>
+      <c r="B13">
+        <v>1161817.3799999999</v>
+      </c>
+      <c r="C13">
+        <v>2657</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A14" s="1">
+        <v>40878</v>
+      </c>
+      <c r="B14">
+        <v>518192.79</v>
+      </c>
+      <c r="C14">
+        <v>778</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8764972-02A7-4617-94DD-157B8766CF6E}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="15.3046875" customWidth="1"/>
+    <col min="2" max="2" width="12.53515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2">
+        <v>7308391.5539999995</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>285446.34000000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4">
+        <v>265545.90000000002</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5">
+        <v>228867.14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6">
+        <v>209024.05</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>138521.31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
+        <v>61577.11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <v>56443.95</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10">
+        <v>41196.339999999997</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>38378.33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6DD4CF2-AF02-4EDD-8F29-8B589E7DCA63}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="20.61328125" customWidth="1"/>
+    <col min="2" max="2" width="20.84375" customWidth="1"/>
+    <col min="3" max="3" width="17.921875" customWidth="1"/>
+    <col min="4" max="4" width="12.921875" customWidth="1"/>
+    <col min="5" max="5" width="16.3828125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="18.45" x14ac:dyDescent="0.5">
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="20.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="4">
+        <f>KPI_Summary!B2</f>
+        <v>8911407.9039999992</v>
+      </c>
+      <c r="B2" s="3">
+        <f>KPI_Summary!B3</f>
+        <v>18532</v>
+      </c>
+      <c r="C2" s="3">
+        <f>KPI_Summary!B4</f>
+        <v>4338</v>
+      </c>
+      <c r="D2" s="4">
+        <f>KPI_Summary!B5</f>
+        <v>480.86595639974092</v>
+      </c>
+      <c r="E2" s="5">
+        <f>KPI_Summary!B6</f>
+        <v>0.65583218072844629</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>